<commit_message>
Add bank-statement category auto-detection
</commit_message>
<xml_diff>
--- a/Tests/CashRunwayCoreTests/Fixtures/privatbank.xlsx
+++ b/Tests/CashRunwayCoreTests/Fixtures/privatbank.xlsx
@@ -77,7 +77,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Shopping</t>
+          <t>Супермаркети та продукти</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -123,7 +123,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Transfer</t>
+          <t>Зарахування</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -169,7 +169,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Car rental</t>
+          <t>АЗС</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">

</xml_diff>

<commit_message>
Address bank category detection review
</commit_message>
<xml_diff>
--- a/Tests/CashRunwayCoreTests/Fixtures/privatbank.xlsx
+++ b/Tests/CashRunwayCoreTests/Fixtures/privatbank.xlsx
@@ -87,11 +87,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Temu</t>
+          <t>Synthetic Market</t>
         </is>
       </c>
       <c r="E3">
-        <v>-499.99</v>
+        <v>-123.45</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -99,7 +99,7 @@
         </is>
       </c>
       <c r="G3">
-        <v>-499.99</v>
+        <v>-123.45</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
@@ -107,7 +107,7 @@
         </is>
       </c>
       <c r="I3">
-        <v>10000.00</v>
+        <v>9876.55</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -133,11 +133,11 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Новосад С.</t>
+          <t>Тестовий Відправник</t>
         </is>
       </c>
       <c r="E4">
-        <v>2800.00</v>
+        <v>250.00</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
@@ -145,7 +145,7 @@
         </is>
       </c>
       <c r="G4">
-        <v>2800.00</v>
+        <v>250.00</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -153,7 +153,7 @@
         </is>
       </c>
       <c r="I4">
-        <v>10500.00</v>
+        <v>10126.55</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -179,11 +179,11 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SIXT, Monaco</t>
+          <t>Sample Fuel Rental</t>
         </is>
       </c>
       <c r="E5">
-        <v>-2041.88</v>
+        <v>-67.89</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
@@ -191,7 +191,7 @@
         </is>
       </c>
       <c r="G5">
-        <v>-50.00</v>
+        <v>-2.00</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -199,7 +199,7 @@
         </is>
       </c>
       <c r="I5">
-        <v>8000.00</v>
+        <v>9808.66</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>

</xml_diff>